<commit_message>
Adicionado exercicio avançado de função SE dentro do arquivo exercicio_temperatura
</commit_message>
<xml_diff>
--- a/Excel/aula_6_se/exercicio_temperatura.xlsx
+++ b/Excel/aula_6_se/exercicio_temperatura.xlsx
@@ -3,10 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Folha1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="se_basico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="se_avancado" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Paciente</t>
   </si>
@@ -34,6 +35,9 @@
   </si>
   <si>
     <t>Carlo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agora, preciso ver se a temperatura está abaixo de 39 ou acima de 39</t>
   </si>
 </sst>
 </file>
@@ -68,8 +72,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -593,7 +600,7 @@
         <v>37.5</v>
       </c>
       <c r="C2" t="str">
-        <f>IF(B2&gt;37.5,"Chamar o médico","Monitorar")</f>
+        <f t="shared" ref="C2:C4" si="0">IF(B2&gt;37.5,"Chamar o médico","Monitorar")</f>
         <v>Monitorar</v>
       </c>
     </row>
@@ -605,7 +612,7 @@
         <v>38</v>
       </c>
       <c r="C3" t="str">
-        <f>IF(B3&gt;37.5,"Chamar o médico","Monitorar")</f>
+        <f t="shared" si="0"/>
         <v xml:space="preserve">Chamar o médico</v>
       </c>
     </row>
@@ -617,16 +624,81 @@
         <v>36</v>
       </c>
       <c r="C4" t="str">
-        <f>IF(B4&gt;37.5,"Chamar o médico","Monitorar")</f>
+        <f t="shared" si="0"/>
         <v>Monitorar</v>
       </c>
-    </row>
-    <row r="5" ht="14.25">
-      <c r="C5"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000008" footer="0.31496062000000008"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col bestFit="1" min="2" max="2" width="11.8515625"/>
+    <col bestFit="1" min="3" max="3" width="15.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>37.5</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <f>IF(B4&gt;37.5,IF(B4&lt;39,"Antitermico","Chamar Emergência"),"Monitorar")</f>
+        <v>Monitorar</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>38</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <f>IF(B5&gt;37.5,IF(B5&lt;39,"Antitermico","Chamar Emergência"),"Monitorar")</f>
+        <v>Antitermico</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>39</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <f>IF(B6&gt;37.5,IF(B6&lt;39,"Antitermico","Chamar Emergência"),"Monitorar")</f>
+        <v xml:space="preserve">Chamar Emergência</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>

</xml_diff>